<commit_message>
arreglo nombre de desarrollador, nombre del archivo conforme a estandar, y hojas de logs y code review
</commit_message>
<xml_diff>
--- a/templates/TDD.xlsx
+++ b/templates/TDD.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mvidaurre\Desktop\RPA\uatAcelerator\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B81A910-B54B-41DB-9518-250DA1430E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2CA116F-99F6-431B-BB2D-0A1EE2DDF997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="3" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cover" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,8 @@
     <sheet name="Escenario_Single" sheetId="4" r:id="rId4"/>
     <sheet name="Escenario_Complejo" sheetId="5" r:id="rId5"/>
     <sheet name="Recomendaciones" sheetId="6" r:id="rId6"/>
+    <sheet name="LOG" sheetId="8" r:id="rId7"/>
+    <sheet name="Code Review" sheetId="7" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -269,7 +271,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="63">
   <si>
     <t xml:space="preserve"> Escenario {{ numero }}</t>
   </si>
@@ -437,13 +439,34 @@
   </si>
   <si>
     <t xml:space="preserve"> Recomendaciones - Posibles escenarios para pensar</t>
+  </si>
+  <si>
+    <t>DATE TIME</t>
+  </si>
+  <si>
+    <t>BOT NAME</t>
+  </si>
+  <si>
+    <t>TASK NAME</t>
+  </si>
+  <si>
+    <t>STATUS</t>
+  </si>
+  <si>
+    <t>DESCRIPTION</t>
+  </si>
+  <si>
+    <t>Log de escenario {{ numero }}</t>
+  </si>
+  <si>
+    <t>Code Review</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -559,8 +582,15 @@
       <name val="Tahoma"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -607,6 +637,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFED7D31"/>
+        <bgColor rgb="FFED7D31"/>
       </patternFill>
     </fill>
   </fills>
@@ -738,7 +774,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="56">
+  <cellXfs count="60">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -856,6 +892,9 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -878,8 +917,15 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1185,21 +1231,21 @@
       </c>
     </row>
     <row r="6" spans="2:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="45" t="s">
+      <c r="B6" s="46" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
-      <c r="H6" s="45"/>
-      <c r="I6" s="45"/>
-      <c r="J6" s="45"/>
-      <c r="K6" s="45"/>
-      <c r="L6" s="45"/>
-      <c r="M6" s="45"/>
-      <c r="N6" s="45"/>
+      <c r="C6" s="46"/>
+      <c r="D6" s="46"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
+      <c r="H6" s="46"/>
+      <c r="I6" s="46"/>
+      <c r="J6" s="46"/>
+      <c r="K6" s="46"/>
+      <c r="L6" s="46"/>
+      <c r="M6" s="46"/>
+      <c r="N6" s="46"/>
     </row>
     <row r="7" spans="2:14" ht="21" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="28" t="s">
@@ -1234,13 +1280,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A2" s="46" t="s">
+      <c r="A2" s="47" t="s">
         <v>18</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
     </row>
     <row r="3" spans="1:5" s="6" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
@@ -1249,47 +1295,47 @@
       <c r="C3" s="23"/>
     </row>
     <row r="4" spans="1:5" s="5" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="49" t="s">
+      <c r="A4" s="50" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="50"/>
+      <c r="B4" s="51"/>
       <c r="C4" s="20" t="str">
         <f ca="1">MID(CELL("filename"),FIND("[",CELL("filename"))+1,FIND("]",CELL("filename"))-FIND("[",CELL("filename"))-1)</f>
         <v>TDD.xlsx</v>
       </c>
     </row>
     <row r="5" spans="1:5" s="5" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="49" t="s">
+      <c r="A5" s="50" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="50"/>
+      <c r="B5" s="51"/>
       <c r="C5" s="20" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:5" s="5" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="49" t="s">
+      <c r="A6" s="50" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="50"/>
+      <c r="B6" s="51"/>
       <c r="C6" s="20" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:5" s="5" customFormat="1" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="49" t="s">
+      <c r="A7" s="50" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="50"/>
+      <c r="B7" s="51"/>
       <c r="C7" s="20" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:5" s="5" customFormat="1" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="49" t="s">
+      <c r="A8" s="50" t="s">
         <v>26</v>
       </c>
-      <c r="B8" s="50"/>
+      <c r="B8" s="51"/>
       <c r="C8" s="22" t="s">
         <v>17</v>
       </c>
@@ -1325,16 +1371,16 @@
       <c r="C12" s="24" t="s">
         <v>34</v>
       </c>
-      <c r="D12" s="51" t="s">
+      <c r="D12" s="52" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="52"/>
+      <c r="E12" s="53"/>
     </row>
     <row r="13" spans="1:5" ht="15" x14ac:dyDescent="0.25">
       <c r="A13"/>
       <c r="C13" s="21"/>
-      <c r="D13" s="48"/>
-      <c r="E13" s="47"/>
+      <c r="D13" s="49"/>
+      <c r="E13" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -1459,14 +1505,14 @@
       </c>
     </row>
     <row r="6" spans="1:6" s="17" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="54"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
     </row>
     <row r="7" spans="1:6" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="30"/>
@@ -1573,14 +1619,14 @@
       <c r="B5" s="16"/>
     </row>
     <row r="6" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="54" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="54"/>
-      <c r="C6" s="54"/>
-      <c r="D6" s="54"/>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
+      <c r="B6" s="55"/>
+      <c r="C6" s="55"/>
+      <c r="D6" s="55"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
     </row>
     <row r="7" spans="1:6" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="30"/>
@@ -1654,7 +1700,7 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="55" t="s">
+      <c r="A2" s="45" t="s">
         <v>54</v>
       </c>
     </row>
@@ -1663,4 +1709,84 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <legacyDrawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F031A64F-9808-4781-A29A-0ADC235D2F23}">
+  <dimension ref="A1:E3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="2" max="2" width="11.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" customWidth="1"/>
+    <col min="4" max="4" width="8.85546875" customWidth="1"/>
+    <col min="5" max="5" width="50.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="56" t="s">
+        <v>61</v>
+      </c>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="57"/>
+      <c r="B2" s="57"/>
+      <c r="C2" s="57"/>
+      <c r="D2" s="57"/>
+      <c r="E2" s="57"/>
+    </row>
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="58" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" s="59" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="58" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="59" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="58" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{336B5D8E-7DE7-40B0-AA04-4D1F39F4D744}">
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="5" max="5" width="58.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="56" t="s">
+        <v>62</v>
+      </c>
+      <c r="B1" s="56"/>
+      <c r="C1" s="56"/>
+      <c r="D1" s="56"/>
+      <c r="E1" s="56"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>